<commit_message>
change label size for Jpsi
</commit_message>
<xml_diff>
--- a/NEW/python/data.xlsx
+++ b/NEW/python/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwpark\Desktop\git\Belle2_script\NEW\python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D5FAEF-E626-4780-AE04-939D85B8AD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57FE25D-6182-4017-8725-B9FC49BA5E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -367,13 +367,13 @@
   <sheetData>
     <row r="1" spans="1:31">
       <c r="A1" s="1">
-        <v>9.0730730000000008</v>
+        <v>9.0489660000000001</v>
       </c>
       <c r="B1" s="1">
-        <v>2.5584199999999999</v>
+        <v>2.5516540000000001</v>
       </c>
       <c r="C1" s="1">
-        <v>1.22095</v>
+        <v>1.2177230000000001</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -406,13 +406,13 @@
     </row>
     <row r="2" spans="1:31">
       <c r="A2" s="1">
-        <v>0.15636700000000001</v>
+        <v>0.15595400000000001</v>
       </c>
       <c r="B2" s="1">
-        <v>4.6268890000000003</v>
+        <v>4.6148610000000003</v>
       </c>
       <c r="C2" s="1">
-        <v>1.1136619999999999</v>
+        <v>1.1107670000000001</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -445,13 +445,13 @@
     </row>
     <row r="3" spans="1:31">
       <c r="A3" s="1">
-        <v>0.16438700000000001</v>
+        <v>0.16395100000000001</v>
       </c>
       <c r="B3" s="1">
-        <v>0.33014300000000002</v>
+        <v>0.32928600000000002</v>
       </c>
       <c r="C3" s="1">
-        <v>4.5813269999999999</v>
+        <v>4.5693770000000002</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>

</xml_diff>